<commit_message>
Todo el curso sobre Excel en OneDrive: practicas 3.1, 3.2, 4.1 y 4.2 sin SharePoint, nuevos libros de datos y presentaciones alineadas
</commit_message>
<xml_diff>
--- a/DATOS/SolicitudesVacaciones_OneDrive.xlsx
+++ b/DATOS/SolicitudesVacaciones_OneDrive.xlsx
@@ -126,18 +126,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Solicitudes" displayName="Solicitudes" ref="A1:I6" headerRowCount="1">
-  <autoFilter ref="A1:I6"/>
-  <tableColumns count="9">
-    <tableColumn id="1" name="Title"/>
-    <tableColumn id="2" name="FechaInicio"/>
-    <tableColumn id="3" name="FechaFin"/>
-    <tableColumn id="4" name="Dias"/>
-    <tableColumn id="5" name="Tipo"/>
-    <tableColumn id="6" name="Estado"/>
-    <tableColumn id="7" name="Solicitante"/>
-    <tableColumn id="8" name="Aprobador"/>
-    <tableColumn id="9" name="Comentarios"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Solicitudes" displayName="Solicitudes" ref="A1:J6" headerRowCount="1">
+  <autoFilter ref="A1:J6"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="2" name="Title"/>
+    <tableColumn id="3" name="FechaInicio"/>
+    <tableColumn id="4" name="FechaFin"/>
+    <tableColumn id="5" name="Dias"/>
+    <tableColumn id="6" name="Tipo"/>
+    <tableColumn id="7" name="Estado"/>
+    <tableColumn id="8" name="Solicitante"/>
+    <tableColumn id="9" name="Aprobador"/>
+    <tableColumn id="10" name="Comentarios"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -432,279 +433,310 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>FechaInicio</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>FechaFin</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Dias</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Solicitante</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Aprobador</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Comentarios</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>SOL-20260801090000</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Vacaciones de verano</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>10</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Vacaciones</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Aprobada</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>ana.lopez@contoso.com</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>carmen.ruiz@contoso.com</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Disfrútalas</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>SOL-20260902101500</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mudanza</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>2</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Asuntos propios</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>ana.lopez@contoso.com</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>carmen.ruiz@contoso.com</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>SOL-20260903113000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Curso de Power BI</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Formación</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>luis.garcia@contoso.com</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>carmen.ruiz@contoso.com</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Formación interna</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>SOL-20260904124500</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Puente de diciembre</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>2026-12-07</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>2026-12-08</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Vacaciones</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>luis.garcia@contoso.com</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>carmen.ruiz@contoso.com</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>SOL-20260905140000</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Cita médica</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Asuntos propios</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Rechazada</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>ana.lopez@contoso.com</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>carmen.ruiz@contoso.com</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Coincide con cierre de mes</t>
         </is>

</xml_diff>